<commit_message>
Drop RNOLR2630006R (Electric Vehicle_30) everywhere — no file, no registry entry
Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0161jaxJZTksz7q1T7aevp9F
</commit_message>
<xml_diff>
--- a/lr-radio-30s-isci-map.xlsx
+++ b/lr-radio-30s-isci-map.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1653,58 +1653,6 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>RNOLR2630006R</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>Electric Vehicle_30</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>Radio</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>RNO</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="n">
-        <v>30</v>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>Auto Accidents</t>
-        </is>
-      </c>
-      <c r="H22" s="3" t="inlineStr"/>
-      <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t>17%</t>
-        </is>
-      </c>
-      <c r="J22" s="3" t="inlineStr">
-        <is>
-          <t>NO DRIVE LINK in traffic sheet - chase down</t>
-        </is>
-      </c>
-      <c r="K22" s="3" t="inlineStr">
-        <is>
-          <t>LRRO31208</t>
-        </is>
-      </c>
-      <c r="L22" s="3" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>